<commit_message>
Add Why this priority column to IG Prioritization sheet
Explain P0–P3 assignment for each product using adoption, core journey,
complexity, support dependency, and documentation gap signals.

Co-authored-by: payu-docs <palgunams21@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs-coverage-tracker/PayU_Product_Documentation_Coverage_Tracker.xlsx
+++ b/docs-coverage-tracker/PayU_Product_Documentation_Coverage_Tracker.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Product Documentation Inventory'!$A$1:$AG$88</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'IG Prioritization'!$A$4:$J$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'IG Prioritization'!$A$4:$K$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Coverage Scoring'!$A$17:$J$104</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Coverage by Category'!$A$3:$G$24</definedName>
   </definedNames>
@@ -955,7 +955,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source of truth: PayU Developer Documentation repository (docs/, reference/, recipes/, custom_pages/). Generated: 2026-08-11 12:44 UTC. DevEx goal: Enable developers to successfully integrate PayU products without requiring support intervention.</t>
+          <t>Source of truth: PayU Developer Documentation repository (docs/, reference/, recipes/, custom_pages/). Generated: 2026-08-11 12:50 UTC. DevEx goal: Enable developers to successfully integrate PayU products without requiring support intervention.</t>
         </is>
       </c>
     </row>
@@ -19380,19 +19380,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:K91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19402,15 +19403,15 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1">
+    <row r="2" ht="48" customHeight="1">
       <c r="A2" s="19" t="inlineStr">
         <is>
-          <t>Rule: Recommend a dedicated Integration Guide only where it provides meaningful DevEx value (core journey, high complexity, high support dependency, or revenue-critical). Plugins/utilities/ops products may use install guides or API maps instead.</t>
+          <t>Rule: Recommend a dedicated Integration Guide only where it provides meaningful DevEx value (core journey, high complexity, high support dependency, or revenue-critical). Plugins/utilities/ops products may use install guides or API maps instead. Priority basis: P0 = must have IG now (core/high-support); P1 = next (high DevEx/vertical impact); P2 = later; P3 = low / no dedicated IG needed. See 'Why this priority' for each row.</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="4">
+    <row r="4" ht="36" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Product Name</t>
@@ -19433,36 +19434,41 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
+          <t>Why this priority</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
           <t>Merchant Adoption Signal</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Core Payment Journey</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Developer Complexity</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Support Dependency Risk</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>Existing Gap Severity</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>Rationale / Action</t>
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="48" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Android CheckoutPro SDK</t>
@@ -19485,36 +19491,41 @@
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; moderate complexity; high support dependency without a clear IG; docs relatively stronger (80.0%).</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>Primary Android integration path; ensure Integration Guide covers offers/TPV/sample app and keep troubleshooting current.</t>
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="48" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Checkout Plus (ICP / Bolt Checkout)</t>
@@ -19537,36 +19548,41 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; on the core payment journey; moderate complexity; high support dependency without a clear IG; docs relatively stronger (80.0%).</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>Consolidate Checkout Plus / ICP / Bolt naming; expand Integration Guide with testing, go-live, troubleshooting; reduce reliance on ASK AI duplicate page.</t>
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="48" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Cross-Border Payments Import (PACB)</t>
@@ -19589,36 +19605,41 @@
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; on the core payment journey; high developer complexity; high support dependency without a clear IG; large doc gap (50.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>Dedicated Integration Guide covering card/UPI/NB, LRS, virtual accounts, subscriptions-CB, and onboarding; standardize CB/PACB/Import naming.</t>
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="48" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>EMI / Cardless EMI</t>
@@ -19641,36 +19662,41 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (60.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr">
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J8" s="8" t="inlineStr">
+      <c r="K8" s="8" t="inlineStr">
         <is>
           <t>Create dedicated EMI Integration Guide covering hosted/MH/S2S + NTB flow; link Affordability suite.</t>
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Merchant Hosted Checkout (Custom / Seamless)</t>
@@ -19693,36 +19719,41 @@
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; on the core payment journey; moderate complexity; high support dependency without a clear IG; docs relatively stronger (95.0%).</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H9" s="8" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I9" s="8" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J9" s="8" t="inlineStr">
+      <c r="K9" s="8" t="inlineStr">
         <is>
           <t>Publish a single merchant-journey Integration Guide that stitches payment-method pages (cards/NB/UPI/wallets/EMI/BNPL), hashing, webhooks, verify payment, and go-live into one narrative.</t>
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="48" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Offer Engine / Offers</t>
@@ -19745,36 +19776,41 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (60.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J10" s="8" t="inlineStr">
+      <c r="K10" s="8" t="inlineStr">
         <is>
           <t>Ship Offer Engine Integration Guide (dashboard create → apply at checkout → validate → settle/refund). ASK AI duplicate should redirect to canonical.</t>
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Partner Merchant Onboarding (API / OAuth)</t>
@@ -19797,36 +19833,41 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; high developer complexity; high support dependency without a clear IG; docs relatively stronger (100.0%).</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I11" s="8" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J11" s="8" t="inlineStr">
+      <c r="K11" s="8" t="inlineStr">
         <is>
           <t>Finalize internal-review partner overview as canonical Integration Guide; merge duplicate Partner Integration - Merchant Onboarding APIs tree; fix ParTner folder casing.</t>
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="48" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>PayU Hosted Checkout (Prebuilt)</t>
@@ -19849,36 +19890,41 @@
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; on the core payment journey; moderate complexity; high support dependency without a clear IG; docs relatively stronger (90.0%).</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr">
+      <c r="J12" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J12" s="8" t="inlineStr">
+      <c r="K12" s="8" t="inlineStr">
         <is>
           <t>Strengthen dedicated end-to-end Integration Guide with go-live checklist, troubleshooting, and clearer path from hash → request → callback → verify payment.</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="48" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>PayU Payouts</t>
@@ -19901,36 +19947,41 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; on the core payment journey; moderate complexity; high support dependency without a clear IG; docs relatively stronger (80.0%).</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H13" s="8" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I13" s="8" t="inlineStr">
+      <c r="J13" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J13" s="8" t="inlineStr">
+      <c r="K13" s="8" t="inlineStr">
         <is>
           <t>Elevate Single Transfer + Smart Send + Beneficiary + Webhooks into a master Payouts Integration Guide with go-live; remove releasepending- filename residue from Pay to Phone.</t>
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Payment Links</t>
@@ -19953,36 +20004,41 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; on the core payment journey; moderate complexity; high support dependency without a clear IG; moderate doc gap (70.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr">
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J14" s="8" t="inlineStr">
+      <c r="K14" s="8" t="inlineStr">
         <is>
           <t>Ship a dedicated Payment Links Integration Guide covering dashboard + API creation, webhooks, TPV variant, WhatsApp EPL, and go-live.</t>
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="48" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Server-to-Server (S2S) Checkout</t>
@@ -20005,36 +20061,41 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; on the core payment journey; high developer complexity; high support dependency without a clear IG; docs relatively stronger (95.0%).</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="I15" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J15" s="8" t="inlineStr">
+      <c r="K15" s="8" t="inlineStr">
         <is>
           <t>Create a unified S2S Integration Guide covering classic, decoupled, and direct-authorization flows with decision tree, error handling, and go-live checklist.</t>
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="48" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Split Settlements (Aggregator / Marketplace)</t>
@@ -20057,36 +20118,41 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; on the core payment journey; high developer complexity; high support dependency without a clear IG; moderate doc gap (70.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr">
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J16" s="8" t="inlineStr">
+      <c r="K16" s="8" t="inlineStr">
         <is>
           <t>Fix folder typo split-settlments; publish marketplace Integration Guide (parent/child onboarding → split during/after txn → refunds/settlements).</t>
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="48" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Subscriptions / Recurring Payments</t>
@@ -20109,36 +20175,41 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; on the core payment journey; high developer complexity; high support dependency without a clear IG; moderate doc gap (60.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="I17" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I17" s="8" t="inlineStr">
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J17" s="8" t="inlineStr">
+      <c r="K17" s="8" t="inlineStr">
         <is>
           <t>MUST have a single Integration Guide that unifies SI/Recurring/Subscriptions naming, consent→PDN→recurring, UPI AutoPay, eNACH, and cards; retire ASK AI duplicate into canonical.</t>
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="48" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>Third-Party Verification (TPV)</t>
@@ -20161,36 +20232,41 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; high developer complexity; high support dependency without a clear IG; large doc gap (35.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="I18" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
+      <c r="J18" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J18" s="8" t="inlineStr">
+      <c r="K18" s="8" t="inlineStr">
         <is>
           <t>Create TPV Integration Guide covering Hosted/MH/S2S/Payment Link/NEFT; consolidate dispersed API JSON (tpv-*.json) into reference IA; merge ASK AI guides.</t>
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="48" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Tokenization / Save Cards (Vault)</t>
@@ -20213,36 +20289,41 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; high developer complexity; high support dependency without a clear IG; large doc gap (30.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I19" s="8" t="inlineStr">
+      <c r="J19" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J19" s="8" t="inlineStr">
+      <c r="K19" s="8" t="inlineStr">
         <is>
           <t>Dedicated Integration Guide for Models 1–3 + push tokenization; critical for PCI-reducing integrations and recurring.</t>
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="48" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>iOS CheckoutPro SDK</t>
@@ -20265,36 +20346,41 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
+          <t>P0 — must have a dedicated Integration Guide immediately because of high merchant adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (60.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I20" s="8" t="inlineStr">
+      <c r="J20" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J20" s="8" t="inlineStr">
+      <c r="K20" s="8" t="inlineStr">
         <is>
           <t>Primary iOS path; add explicit go-live checklist and changelog parity with Android.</t>
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="48" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Affordability Widget</t>
@@ -20317,36 +20403,41 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (50.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I21" s="8" t="inlineStr">
+      <c r="J21" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J21" s="8" t="inlineStr">
+      <c r="K21" s="8" t="inlineStr">
         <is>
           <t>Dedicated JS/React widget Integration Guide with plugin variants (Shopify/Woo).</t>
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="48" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Agentic Commerce Suite</t>
@@ -20369,36 +20460,41 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (30.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H22" s="8" t="inlineStr">
+      <c r="I22" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I22" s="8" t="inlineStr">
+      <c r="J22" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J22" s="8" t="inlineStr">
+      <c r="K22" s="8" t="inlineStr">
         <is>
           <t>Emerging DevEx surface — invest in Integration Guide covering ChatGPT merchant app and agent-compatible checkout.</t>
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="48" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Android Core SDK</t>
@@ -20421,36 +20517,41 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (60.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H23" s="8" t="inlineStr">
+      <c r="I23" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I23" s="8" t="inlineStr">
+      <c r="J23" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J23" s="8" t="inlineStr">
+      <c r="K23" s="8" t="inlineStr">
         <is>
           <t>Document decision: CheckoutPro vs Core; Integration Guide should include TPV and web services.</t>
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="48" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Android POS SDK</t>
@@ -20473,36 +20574,41 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (45.5% coverage).</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H24" s="8" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I24" s="8" t="inlineStr">
+      <c r="J24" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J24" s="8" t="inlineStr">
+      <c r="K24" s="8" t="inlineStr">
         <is>
           <t>Expand SDK Integration Guide with sample app walkthrough, error handling, testing, and changelog.</t>
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="48" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Apple Pay</t>
@@ -20525,36 +20631,41 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (40.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H25" s="8" t="inlineStr">
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I25" s="8" t="inlineStr">
+      <c r="J25" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J25" s="8" t="inlineStr">
+      <c r="K25" s="8" t="inlineStr">
         <is>
           <t>Keep prerequisites + Hosted/MH/session/UI as one Integration Guide with Apple certification/testing steps.</t>
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="48" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>BBPS Connect Agent</t>
@@ -20577,36 +20688,41 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; on the core payment journey; moderate complexity; high support dependency without a clear IG; large doc gap (40.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H26" s="8" t="inlineStr">
+      <c r="I26" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I26" s="8" t="inlineStr">
+      <c r="J26" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J26" s="8" t="inlineStr">
+      <c r="K26" s="8" t="inlineStr">
         <is>
           <t>Expand Integration Guide with auth, bill fetch/pay, complaints, sandbox, error catalog.</t>
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="48" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>BNPL / Pay Later</t>
@@ -20629,36 +20745,41 @@
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (50.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H27" s="8" t="inlineStr">
+      <c r="I27" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I27" s="8" t="inlineStr">
+      <c r="J27" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J27" s="8" t="inlineStr">
+      <c r="K27" s="8" t="inlineStr">
         <is>
           <t>Complete Integration Guide for Link &amp; Pay + quick checkout with testing and go-live.</t>
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="48" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>CommercePro Checkout (Checkout Express)</t>
@@ -20681,36 +20802,41 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; on the core payment journey; moderate complexity; high support dependency without a clear IG; docs relatively stronger (80.0%).</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G28" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H28" s="8" t="inlineStr">
+      <c r="I28" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I28" s="8" t="inlineStr">
+      <c r="J28" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J28" s="8" t="inlineStr">
+      <c r="K28" s="8" t="inlineStr">
         <is>
           <t>Unify CommercePro vs Checkout Express naming; add dedicated go-live + troubleshooting; clarify relationship to plugin CommercePro pages.</t>
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="48" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Dynamic Currency Conversion / International Payments</t>
@@ -20733,36 +20859,41 @@
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (55.6% coverage).</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H29" s="8" t="inlineStr">
+      <c r="I29" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I29" s="8" t="inlineStr">
+      <c r="J29" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J29" s="8" t="inlineStr">
+      <c r="K29" s="8" t="inlineStr">
         <is>
           <t>Unify DCC vs International Payments naming; clarify MCP (multi-currency pricing) vs MCP (Model Context Protocol) collision in docs IA.</t>
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="48" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>Dynamic Storefront QR (DBQR)</t>
@@ -20785,36 +20916,41 @@
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (20.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G30" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H30" s="8" t="inlineStr">
+      <c r="I30" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I30" s="8" t="inlineStr">
+      <c r="J30" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J30" s="8" t="inlineStr">
+      <c r="K30" s="8" t="inlineStr">
         <is>
           <t>Publish a dedicated Integration Guide; resolve DBQR / Offline DBQR / Dynamic Bharat QR naming; surface ASK AI offline-dbqr content into canonical docs.</t>
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="48" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Flutter CheckoutPro SDK</t>
@@ -20837,36 +20973,41 @@
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (60.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H31" s="8" t="inlineStr">
+      <c r="I31" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I31" s="8" t="inlineStr">
+      <c r="J31" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J31" s="8" t="inlineStr">
+      <c r="K31" s="8" t="inlineStr">
         <is>
           <t>Add FAQs/troubleshooting; version history exists — promote as changelog.</t>
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="48" customHeight="1">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>Java SDK</t>
@@ -20889,36 +21030,41 @@
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (66.7% coverage).</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G32" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H32" s="8" t="inlineStr">
+      <c r="I32" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I32" s="8" t="inlineStr">
+      <c r="J32" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J32" s="8" t="inlineStr">
+      <c r="K32" s="8" t="inlineStr">
         <is>
           <t>Upgrade from single-page SDK note to full Integration Guide (install, auth, payment sample, verify, errors, changelog) for high-usage languages.</t>
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" ht="48" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Merchant Wallet</t>
@@ -20941,36 +21087,41 @@
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; on the core payment journey; high developer complexity; high support dependency without a clear IG; large doc gap (40.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G33" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H33" s="8" t="inlineStr">
+      <c r="I33" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I33" s="8" t="inlineStr">
+      <c r="J33" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J33" s="8" t="inlineStr">
+      <c r="K33" s="8" t="inlineStr">
         <is>
           <t>Integration Guides for Closed-Loop vs Open/Semi-Closed issuance journeys; document callbacks/status codes clearly.</t>
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="48" customHeight="1">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>Mutual Fund Payments (WealthTech)</t>
@@ -20993,36 +21144,41 @@
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (30.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G34" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H34" s="8" t="inlineStr">
+      <c r="I34" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I34" s="8" t="inlineStr">
+      <c r="J34" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J34" s="8" t="inlineStr">
+      <c r="K34" s="8" t="inlineStr">
         <is>
           <t>Align Mutual Fund Payments guide naming with Wealth Tech API category; Integration Guide covering eNACH + UPI AutoPay.</t>
         </is>
       </c>
     </row>
-    <row r="35">
+    <row r="35" ht="48" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>Native OTP Flow</t>
@@ -21045,36 +21201,41 @@
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (30.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F35" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H35" s="8" t="inlineStr">
+      <c r="I35" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I35" s="8" t="inlineStr">
+      <c r="J35" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J35" s="8" t="inlineStr">
+      <c r="K35" s="8" t="inlineStr">
         <is>
           <t>Clarify Native OTP Flow (web/API) vs Native OTP Assist mobile SDKs; ship Integration Guide for card/debit/cardless EMI.</t>
         </is>
       </c>
     </row>
-    <row r="36">
+    <row r="36" ht="48" customHeight="1">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>Node.js SDK</t>
@@ -21097,36 +21258,41 @@
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (66.7% coverage).</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F36" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G36" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H36" s="8" t="inlineStr">
+      <c r="I36" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I36" s="8" t="inlineStr">
+      <c r="J36" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J36" s="8" t="inlineStr">
+      <c r="K36" s="8" t="inlineStr">
         <is>
           <t>Upgrade from single-page SDK note to full Integration Guide (install, auth, payment sample, verify, errors, changelog) for high-usage languages.</t>
         </is>
       </c>
     </row>
-    <row r="37">
+    <row r="37" ht="48" customHeight="1">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>PHP SDK</t>
@@ -21149,36 +21315,41 @@
       </c>
       <c r="E37" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (66.7% coverage).</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G37" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H37" s="8" t="inlineStr">
+      <c r="I37" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I37" s="8" t="inlineStr">
+      <c r="J37" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J37" s="8" t="inlineStr">
+      <c r="K37" s="8" t="inlineStr">
         <is>
           <t>Upgrade from single-page SDK note to full Integration Guide (install, auth, payment sample, verify, errors, changelog) for high-usage languages.</t>
         </is>
       </c>
     </row>
-    <row r="38">
+    <row r="38" ht="48" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>POS Terminal Integration</t>
@@ -21201,36 +21372,41 @@
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; on the core payment journey; moderate complexity; high support dependency without a clear IG; large doc gap (40.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G38" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H38" s="8" t="inlineStr">
+      <c r="I38" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I38" s="8" t="inlineStr">
+      <c r="J38" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J38" s="8" t="inlineStr">
+      <c r="K38" s="8" t="inlineStr">
         <is>
           <t>Add end-to-end Integration Guide with device setup, test transactions, error codes, and go-live.</t>
         </is>
       </c>
     </row>
-    <row r="39">
+    <row r="39" ht="48" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Partner Payments Integration</t>
@@ -21253,36 +21429,41 @@
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; high developer complexity; high support dependency without a clear IG; large doc gap (40.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F39" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G39" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H39" s="8" t="inlineStr">
+      <c r="I39" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I39" s="8" t="inlineStr">
+      <c r="J39" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J39" s="8" t="inlineStr">
+      <c r="K39" s="8" t="inlineStr">
         <is>
           <t>Expand Integration Guide for Hosted/UPI S2S/UPI TPV/refunds partner flows.</t>
         </is>
       </c>
     </row>
-    <row r="40">
+    <row r="40" ht="48" customHeight="1">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Pay to Phone</t>
@@ -21305,36 +21486,41 @@
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (60.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F40" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G40" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H40" s="8" t="inlineStr">
+      <c r="I40" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I40" s="8" t="inlineStr">
+      <c r="J40" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J40" s="8" t="inlineStr">
+      <c r="K40" s="8" t="inlineStr">
         <is>
           <t>Rename releasepending- paths; complete Integration Guide for initiation/tracking/configuration.</t>
         </is>
       </c>
     </row>
-    <row r="41">
+    <row r="41" ht="48" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>PayU Remote MCP Server</t>
@@ -21357,36 +21543,41 @@
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (42.9% coverage).</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G41" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H41" s="8" t="inlineStr">
+      <c r="I41" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I41" s="8" t="inlineStr">
+      <c r="J41" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J41" s="8" t="inlineStr">
+      <c r="K41" s="8" t="inlineStr">
         <is>
           <t>Treat current page as Integration Guide seed; add tool catalog, auth (OAuth 2.1), examples, troubleshooting. Disambiguate MCP acronym from Multi-Currency Pricing.</t>
         </is>
       </c>
     </row>
-    <row r="42">
+    <row r="42" ht="48" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>Pre-Authorize / Auth &amp; Capture</t>
@@ -21409,36 +21600,41 @@
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (50.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F42" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G42" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H42" s="8" t="inlineStr">
+      <c r="I42" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I42" s="8" t="inlineStr">
+      <c r="J42" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J42" s="8" t="inlineStr">
+      <c r="K42" s="8" t="inlineStr">
         <is>
           <t>Integration Guide for card pre-auth + capture/cancel with S2S variant.</t>
         </is>
       </c>
     </row>
-    <row r="43">
+    <row r="43" ht="48" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>React Native CheckoutPro SDK</t>
@@ -21461,36 +21657,41 @@
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (70.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G43" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H43" s="8" t="inlineStr">
+      <c r="I43" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I43" s="8" t="inlineStr">
+      <c r="J43" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J43" s="8" t="inlineStr">
+      <c r="K43" s="8" t="inlineStr">
         <is>
           <t>High DevEx impact for cross-platform apps; consolidate duplicate FAQ pages.</t>
         </is>
       </c>
     </row>
-    <row r="44">
+    <row r="44" ht="48" customHeight="1">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>Shopify Plugin</t>
@@ -21513,36 +21714,41 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (71.4% coverage).</t>
+        </is>
+      </c>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F44" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G44" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H44" s="8" t="inlineStr">
+      <c r="I44" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I44" s="8" t="inlineStr">
+      <c r="J44" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J44" s="8" t="inlineStr">
+      <c r="K44" s="8" t="inlineStr">
         <is>
           <t>High-adoption plugin; ensure CommercePro/offers/reconciliation paths are clear; keep Integration Guide as install→configure→go-live.</t>
         </is>
       </c>
     </row>
-    <row r="45">
+    <row r="45" ht="48" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>UPI Bolt SDK (Android/iOS/RN/Flutter/Ionic)</t>
@@ -21565,36 +21771,41 @@
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (50.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G45" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H45" s="8" t="inlineStr">
+      <c r="I45" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I45" s="8" t="inlineStr">
+      <c r="J45" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J45" s="8" t="inlineStr">
+      <c r="K45" s="8" t="inlineStr">
         <is>
           <t>Resolve Ionic/Capacitor/Cordova naming inconsistency; publish one cross-platform UPI Bolt Integration Guide with platform tabs.</t>
         </is>
       </c>
     </row>
-    <row r="46">
+    <row r="46" ht="48" customHeight="1">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>UPI One-Time Mandate (OTM / Reserve Pay)</t>
@@ -21617,36 +21828,41 @@
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (40.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F46" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G46" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H46" s="8" t="inlineStr">
+      <c r="I46" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I46" s="8" t="inlineStr">
+      <c r="J46" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J46" s="8" t="inlineStr">
+      <c r="K46" s="8" t="inlineStr">
         <is>
           <t>Promote OTM to first-class Integration Guide; merge ASK AI upi-otm into canonical docs.</t>
         </is>
       </c>
     </row>
-    <row r="47">
+    <row r="47" ht="48" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>UPI QR</t>
@@ -21669,36 +21885,41 @@
       </c>
       <c r="E47" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; on the core payment journey; moderate complexity; high support dependency without a clear IG; moderate doc gap (65.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="G47" s="8" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H47" s="8" t="inlineStr">
+      <c r="I47" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I47" s="8" t="inlineStr">
+      <c r="J47" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J47" s="8" t="inlineStr">
+      <c r="K47" s="8" t="inlineStr">
         <is>
           <t>Expand Integration Guide with callback/webhook handling, sandbox testing, and go-live steps.</t>
         </is>
       </c>
     </row>
-    <row r="48">
+    <row r="48" ht="48" customHeight="1">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>WhatsApp Payments</t>
@@ -21721,36 +21942,41 @@
       </c>
       <c r="E48" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; large doc gap (40.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G48" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H48" s="8" t="inlineStr">
+      <c r="I48" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I48" s="8" t="inlineStr">
+      <c r="J48" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J48" s="8" t="inlineStr">
+      <c r="K48" s="8" t="inlineStr">
         <is>
           <t>Dedicated Integration Guide for Native P2M + Enhanced Payment Links; clarify Interakt plugin boundary.</t>
         </is>
       </c>
     </row>
-    <row r="49">
+    <row r="49" ht="48" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>WooCommerce Plugin</t>
@@ -21773,36 +21999,41 @@
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (71.4% coverage).</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G49" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H49" s="8" t="inlineStr">
+      <c r="I49" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I49" s="8" t="inlineStr">
+      <c r="J49" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J49" s="8" t="inlineStr">
+      <c r="K49" s="8" t="inlineStr">
         <is>
           <t>High-adoption; reconcile duplicate ASK AI woocommerce guide into canonical docs.</t>
         </is>
       </c>
     </row>
-    <row r="50">
+    <row r="50" ht="48" customHeight="1">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Zion Subscription Automation</t>
@@ -21825,36 +22056,41 @@
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; high developer complexity; high support dependency without a clear IG; large doc gap (50.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G50" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H50" s="8" t="inlineStr">
+      <c r="I50" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I50" s="8" t="inlineStr">
+      <c r="J50" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J50" s="8" t="inlineStr">
+      <c r="K50" s="8" t="inlineStr">
         <is>
           <t>Dedicated Zion Integration Guide (plans, invoices, webhooks lifecycle) with consistent Zion/ZION casing.</t>
         </is>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="48" customHeight="1">
       <c r="A51" s="8" t="inlineStr">
         <is>
           <t>iOS Core SDK</t>
@@ -21877,30 +22113,35 @@
       </c>
       <c r="E51" s="8" t="inlineStr">
         <is>
+          <t>P1 — important next; schedule after P0 core journeys because of medium adoption; moderate complexity; high support dependency without a clear IG; moderate doc gap (60.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F51" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G51" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H51" s="8" t="inlineStr">
+      <c r="I51" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I51" s="8" t="inlineStr">
+      <c r="J51" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J51" s="8" t="inlineStr">
+      <c r="K51" s="8" t="inlineStr">
         <is>
           <t>Cover recurring/TPV; align release notes.</t>
         </is>
@@ -21929,30 +22170,35 @@
       </c>
       <c r="E52" s="8" t="inlineStr">
         <is>
+          <t>P2 — improve later; lower urgency vs core journeys because of lower/niche adoption; moderate complexity; moderate support risk; moderate doc gap (71.4% coverage).</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F52" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G52" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H52" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H52" s="8" t="inlineStr">
+      <c r="I52" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I52" s="8" t="inlineStr">
+      <c r="J52" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J52" s="8" t="inlineStr">
+      <c r="K52" s="8" t="inlineStr">
         <is>
           <t>Maintain install + CommercePro + troubleshooting; Integration Guide valuable for merchants.</t>
         </is>
@@ -21981,30 +22227,35 @@
       </c>
       <c r="E53" s="8" t="inlineStr">
         <is>
+          <t>P2 — improve later; lower urgency vs core journeys because of lower/niche adoption; high developer complexity; moderate support risk; large doc gap (30.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F53" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G53" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H53" s="8" t="inlineStr">
+      <c r="I53" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I53" s="8" t="inlineStr">
+      <c r="J53" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J53" s="8" t="inlineStr">
+      <c r="K53" s="8" t="inlineStr">
         <is>
           <t>Consolidate RewardX, Pay with Rewards/TWID, and Flipkart SuperCoins IA to reduce duplication.</t>
         </is>
@@ -22033,30 +22284,35 @@
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
+          <t>P2 — improve later; lower urgency vs core journeys because of lower/niche adoption; moderate complexity; moderate support risk; large doc gap (36.4% coverage).</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F54" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G54" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H54" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H54" s="8" t="inlineStr">
+      <c r="I54" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I54" s="8" t="inlineStr">
+      <c r="J54" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J54" s="8" t="inlineStr">
+      <c r="K54" s="8" t="inlineStr">
         <is>
           <t>One Integration Guide with web + mobile SDK matrix; promote API map to reference section.</t>
         </is>
@@ -22085,30 +22341,35 @@
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
+          <t>P2 — improve later; lower urgency vs core journeys because of lower/niche adoption; moderate complexity; moderate support risk; moderate doc gap (57.1% coverage).</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F55" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H55" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H55" s="8" t="inlineStr">
+      <c r="I55" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="I55" s="8" t="inlineStr">
+      <c r="J55" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J55" s="8" t="inlineStr">
+      <c r="K55" s="8" t="inlineStr">
         <is>
           <t>Multiple Zoho surfaces (Marketplace/One/Billing/Inventory); recommend one Integration Guide with product matrix.</t>
         </is>
@@ -22137,30 +22398,35 @@
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
+          <t>P1: dedicated IG not the primary ask — medium adoption; moderate doc gap (75.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F56" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H56" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H56" s="8" t="inlineStr">
+      <c r="I56" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I56" s="8" t="inlineStr">
+      <c r="J56" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J56" s="8" t="inlineStr">
+      <c r="K56" s="8" t="inlineStr">
         <is>
           <t>Do not create product IG; instead improve discoverability from checkout IGs (verify payment, BIN, health check).</t>
         </is>
@@ -22189,30 +22455,35 @@
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
+          <t>P1: dedicated IG not the primary ask — medium adoption; moderate doc gap (55.6% coverage).</t>
+        </is>
+      </c>
+      <c r="F57" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F57" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H57" s="8" t="inlineStr">
+      <c r="I57" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I57" s="8" t="inlineStr">
+      <c r="J57" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J57" s="8" t="inlineStr">
+      <c r="K57" s="8" t="inlineStr">
         <is>
           <t>Keep API + webhooks + product-specific refund pages strong; cross-link from every collect product. Dedicated IG not needed beyond current structure.</t>
         </is>
@@ -22241,30 +22512,35 @@
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
+          <t>P1: dedicated IG not the primary ask — medium adoption; moderate doc gap (70.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F58" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F58" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H58" s="8" t="inlineStr">
+      <c r="I58" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I58" s="8" t="inlineStr">
+      <c r="J58" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J58" s="8" t="inlineStr">
+      <c r="K58" s="8" t="inlineStr">
         <is>
           <t>Keep as chapter of Payouts IG rather than separate IG.</t>
         </is>
@@ -22293,30 +22569,35 @@
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
+          <t>P1: dedicated IG not the primary ask — medium adoption; moderate doc gap (70.0% coverage).</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F59" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H59" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H59" s="8" t="inlineStr">
+      <c r="I59" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I59" s="8" t="inlineStr">
+      <c r="J59" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J59" s="8" t="inlineStr">
+      <c r="K59" s="8" t="inlineStr">
         <is>
           <t>Has go-live checklist and test integration — model for other SDKs; dedicated IG optional if pages stay cohesive.</t>
         </is>
@@ -22345,30 +22626,35 @@
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (33.3% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F60" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H60" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H60" s="8" t="inlineStr">
+      <c r="I60" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I60" s="8" t="inlineStr">
+      <c r="J60" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J60" s="8" t="inlineStr">
+      <c r="K60" s="8" t="inlineStr">
         <is>
           <t>Add compliance notes and testing guidance; dedicated IG only if adoption rises.</t>
         </is>
@@ -22397,30 +22683,35 @@
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (40.0% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F61" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H61" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H61" s="8" t="inlineStr">
+      <c r="I61" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I61" s="8" t="inlineStr">
+      <c r="J61" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J61" s="8" t="inlineStr">
+      <c r="K61" s="8" t="inlineStr">
         <is>
           <t>Keep as chapter of BBPS IG; add testing/errors.</t>
         </is>
@@ -22449,30 +22740,35 @@
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; moderate doc gap (71.4% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F62" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H62" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H62" s="8" t="inlineStr">
+      <c r="I62" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I62" s="8" t="inlineStr">
+      <c r="J62" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J62" s="8" t="inlineStr">
+      <c r="K62" s="8" t="inlineStr">
         <is>
           <t>Keep troubleshooting current; dedicated IG low value beyond install guide.</t>
         </is>
@@ -22501,30 +22797,35 @@
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (37.5% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F63" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F63" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H63" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H63" s="8" t="inlineStr">
+      <c r="I63" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I63" s="8" t="inlineStr">
+      <c r="J63" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J63" s="8" t="inlineStr">
+      <c r="K63" s="8" t="inlineStr">
         <is>
           <t>Add FAQs and operational runbooks; Integration Guide not required (ops/API product).</t>
         </is>
@@ -22553,30 +22854,35 @@
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (50.0% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F64" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F64" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H64" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H64" s="8" t="inlineStr">
+      <c r="I64" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I64" s="8" t="inlineStr">
+      <c r="J64" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J64" s="8" t="inlineStr">
+      <c r="K64" s="8" t="inlineStr">
         <is>
           <t>Maintain; lower adoption vs RN/Flutter.</t>
         </is>
@@ -22605,30 +22911,35 @@
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (44.4% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F65" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F65" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H65" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H65" s="8" t="inlineStr">
+      <c r="I65" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I65" s="8" t="inlineStr">
+      <c r="J65" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J65" s="8" t="inlineStr">
+      <c r="K65" s="8" t="inlineStr">
         <is>
           <t>Clarify Collect EFTNET vs Payouts Dashboard EFTNET funding feature.</t>
         </is>
@@ -22657,30 +22968,35 @@
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; moderate doc gap (66.7% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F66" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F66" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H66" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H66" s="8" t="inlineStr">
+      <c r="I66" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I66" s="8" t="inlineStr">
+      <c r="J66" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J66" s="8" t="inlineStr">
+      <c r="K66" s="8" t="inlineStr">
         <is>
           <t>Upgrade from single-page SDK note to full Integration Guide (install, auth, payment sample, verify, errors, changelog) for high-usage languages.</t>
         </is>
@@ -22709,30 +23025,35 @@
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; moderate doc gap (57.1% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F67" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H67" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H67" s="8" t="inlineStr">
+      <c r="I67" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I67" s="8" t="inlineStr">
+      <c r="J67" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J67" s="8" t="inlineStr">
+      <c r="K67" s="8" t="inlineStr">
         <is>
           <t>Cross-links with WhatsApp payments; clarify channel boundary.</t>
         </is>
@@ -22761,30 +23082,35 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (42.9% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F68" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H68" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H68" s="8" t="inlineStr">
+      <c r="I68" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I68" s="8" t="inlineStr">
+      <c r="J68" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J68" s="8" t="inlineStr">
+      <c r="K68" s="8" t="inlineStr">
         <is>
           <t>Clarify Invoice vs Payment Link vs Zion subscription invoices; add FAQs.</t>
         </is>
@@ -22813,30 +23139,35 @@
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (30.0% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F69" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F69" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H69" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H69" s="8" t="inlineStr">
+      <c r="I69" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I69" s="8" t="inlineStr">
+      <c r="J69" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J69" s="8" t="inlineStr">
+      <c r="K69" s="8" t="inlineStr">
         <is>
           <t>Expand Merchant Hosted guide; FAQs and testing checklist recommended.</t>
         </is>
@@ -22865,30 +23196,35 @@
       </c>
       <c r="E70" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (14.3% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F70" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F70" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G70" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H70" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H70" s="8" t="inlineStr">
+      <c r="I70" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I70" s="8" t="inlineStr">
+      <c r="J70" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J70" s="8" t="inlineStr">
+      <c r="K70" s="8" t="inlineStr">
         <is>
           <t>Add clear enablement + dashboard journey; Integration Guide only if API/SDK surface expands.</t>
         </is>
@@ -22917,30 +23253,35 @@
       </c>
       <c r="E71" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; moderate doc gap (71.4% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F71" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G71" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H71" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H71" s="8" t="inlineStr">
+      <c r="I71" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I71" s="8" t="inlineStr">
+      <c r="J71" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J71" s="8" t="inlineStr">
+      <c r="K71" s="8" t="inlineStr">
         <is>
           <t>Add FAQs and troubleshooting for KYC/activation blockers; keep onboarding journey as step-by-step guide (not a classic Integration Guide).</t>
         </is>
@@ -22969,30 +23310,35 @@
       </c>
       <c r="E72" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (50.0% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F72" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G72" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H72" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H72" s="8" t="inlineStr">
+      <c r="I72" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I72" s="8" t="inlineStr">
+      <c r="J72" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J72" s="8" t="inlineStr">
+      <c r="K72" s="8" t="inlineStr">
         <is>
           <t>Clarify boundary vs MobiKwik Wallet APIs; keep testing checklist current.</t>
         </is>
@@ -23021,30 +23367,35 @@
       </c>
       <c r="E73" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (42.9% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F73" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F73" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G73" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H73" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H73" s="8" t="inlineStr">
+      <c r="I73" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I73" s="8" t="inlineStr">
+      <c r="J73" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J73" s="8" t="inlineStr">
+      <c r="K73" s="8" t="inlineStr">
         <is>
           <t>Expand command reference and examples; dedicated IG optional.</t>
         </is>
@@ -23073,30 +23424,35 @@
       </c>
       <c r="E74" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; docs relatively stronger (83.3%). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F74" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F74" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G74" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H74" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H74" s="8" t="inlineStr">
+      <c r="I74" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I74" s="8" t="inlineStr">
+      <c r="J74" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J74" s="8" t="inlineStr">
+      <c r="K74" s="8" t="inlineStr">
         <is>
           <t>Improve module-level how-to consistency (settlements, reports, users); add troubleshooting for common dashboard access issues.</t>
         </is>
@@ -23125,30 +23481,35 @@
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (33.3% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F75" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G75" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H75" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H75" s="8" t="inlineStr">
+      <c r="I75" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I75" s="8" t="inlineStr">
+      <c r="J75" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J75" s="8" t="inlineStr">
+      <c r="K75" s="8" t="inlineStr">
         <is>
           <t>Add setup guide and alert catalog; IG not required.</t>
         </is>
@@ -23177,30 +23538,35 @@
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; high developer complexity; large doc gap (50.0% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F76" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F76" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G76" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H76" s="8" t="inlineStr">
+        <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H76" s="8" t="inlineStr">
+      <c r="I76" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I76" s="8" t="inlineStr">
+      <c r="J76" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J76" s="8" t="inlineStr">
+      <c r="K76" s="8" t="inlineStr">
         <is>
           <t>Keep portal how-tos current; link to API onboarding guides.</t>
         </is>
@@ -23229,30 +23595,35 @@
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; moderate doc gap (66.7% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F77" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G77" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H77" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H77" s="8" t="inlineStr">
+      <c r="I77" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I77" s="8" t="inlineStr">
+      <c r="J77" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J77" s="8" t="inlineStr">
+      <c r="K77" s="8" t="inlineStr">
         <is>
           <t>Upgrade from single-page SDK note to full Integration Guide (install, auth, payment sample, verify, errors, changelog) for high-usage languages.</t>
         </is>
@@ -23281,30 +23652,35 @@
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (44.4% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F78" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G78" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H78" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H78" s="8" t="inlineStr">
+      <c r="I78" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I78" s="8" t="inlineStr">
+      <c r="J78" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J78" s="8" t="inlineStr">
+      <c r="K78" s="8" t="inlineStr">
         <is>
           <t>Document CheckoutPro/CommercePro embedding paths; light Integration Guide optional.</t>
         </is>
@@ -23333,30 +23709,35 @@
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; large doc gap (25.0% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F79" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G79" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H79" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H79" s="8" t="inlineStr">
+      <c r="I79" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I79" s="8" t="inlineStr">
+      <c r="J79" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J79" s="8" t="inlineStr">
+      <c r="K79" s="8" t="inlineStr">
         <is>
           <t>Improve API + dashboard cross-links; Priority Settlements page should link Settlements APIs.</t>
         </is>
@@ -23385,30 +23766,35 @@
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
+          <t>P2: dedicated IG not recommended — lower/niche adoption; moderate doc gap (71.4% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F80" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G80" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H80" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H80" s="8" t="inlineStr">
+      <c r="I80" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I80" s="8" t="inlineStr">
+      <c r="J80" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J80" s="8" t="inlineStr">
+      <c r="K80" s="8" t="inlineStr">
         <is>
           <t>Overview + FAQ sufficient; expand only if support volume warrants.</t>
         </is>
@@ -23437,30 +23823,35 @@
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; large doc gap (28.6% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F81" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G81" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H81" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H81" s="8" t="inlineStr">
+      <c r="I81" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I81" s="8" t="inlineStr">
+      <c r="J81" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J81" s="8" t="inlineStr">
+      <c r="K81" s="8" t="inlineStr">
         <is>
           <t>Keep merchant-specific; do not generalize into public product catalog without product decision.</t>
         </is>
@@ -23489,30 +23880,35 @@
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; moderate doc gap (57.1% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F82" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G82" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H82" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H82" s="8" t="inlineStr">
+      <c r="I82" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I82" s="8" t="inlineStr">
+      <c r="J82" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J82" s="8" t="inlineStr">
+      <c r="K82" s="8" t="inlineStr">
         <is>
           <t>Single-page guide; low priority.</t>
         </is>
@@ -23541,30 +23937,35 @@
       </c>
       <c r="E83" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; large doc gap (22.2% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F83" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G83" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H83" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H83" s="8" t="inlineStr">
+      <c r="I83" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I83" s="8" t="inlineStr">
+      <c r="J83" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J83" s="8" t="inlineStr">
+      <c r="K83" s="8" t="inlineStr">
         <is>
           <t>Docs appear hidden/limited; expand when product is generally available.</t>
         </is>
@@ -23593,30 +23994,35 @@
       </c>
       <c r="E84" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; moderate doc gap (57.1% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F84" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G84" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H84" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H84" s="8" t="inlineStr">
+      <c r="I84" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I84" s="8" t="inlineStr">
+      <c r="J84" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J84" s="8" t="inlineStr">
+      <c r="K84" s="8" t="inlineStr">
         <is>
           <t>Thin docs; expand only with merchant demand.</t>
         </is>
@@ -23645,30 +24051,35 @@
       </c>
       <c r="E85" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; moderate doc gap (57.1% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F85" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G85" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H85" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H85" s="8" t="inlineStr">
+      <c r="I85" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I85" s="8" t="inlineStr">
+      <c r="J85" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J85" s="8" t="inlineStr">
+      <c r="K85" s="8" t="inlineStr">
         <is>
           <t>Installation page present; expand if adoption grows.</t>
         </is>
@@ -23697,30 +24108,35 @@
       </c>
       <c r="E86" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; moderate doc gap (71.4% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F86" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G86" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H86" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H86" s="8" t="inlineStr">
+      <c r="I86" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I86" s="8" t="inlineStr">
+      <c r="J86" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J86" s="8" t="inlineStr">
+      <c r="K86" s="8" t="inlineStr">
         <is>
           <t>Install + troubleshooting adequate for plugin channel.</t>
         </is>
@@ -23749,30 +24165,35 @@
       </c>
       <c r="E87" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; large doc gap (50.0% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F87" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G87" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H87" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H87" s="8" t="inlineStr">
+      <c r="I87" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I87" s="8" t="inlineStr">
+      <c r="J87" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J87" s="8" t="inlineStr">
+      <c r="K87" s="8" t="inlineStr">
         <is>
           <t>Internal docs tooling — maintain configuration page only.</t>
         </is>
@@ -23801,30 +24222,35 @@
       </c>
       <c r="E88" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; large doc gap (42.9% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F88" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F88" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G88" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H88" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H88" s="8" t="inlineStr">
+      <c r="I88" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I88" s="8" t="inlineStr">
+      <c r="J88" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J88" s="8" t="inlineStr">
+      <c r="K88" s="8" t="inlineStr">
         <is>
           <t>Expand dashboard how-to with screenshots and FAQs; dedicated Integration Guide not required (no-code UI product).</t>
         </is>
@@ -23853,30 +24279,35 @@
       </c>
       <c r="E89" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; large doc gap (33.3% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F89" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F89" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G89" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H89" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H89" s="8" t="inlineStr">
+      <c r="I89" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I89" s="8" t="inlineStr">
+      <c r="J89" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J89" s="8" t="inlineStr">
+      <c r="K89" s="8" t="inlineStr">
         <is>
           <t>Rename Sodexo reference to Pluxee; keep as method page under Merchant Hosted.</t>
         </is>
@@ -23905,30 +24336,35 @@
       </c>
       <c r="E90" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; moderate doc gap (71.4% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F90" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F90" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H90" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H90" s="8" t="inlineStr">
+      <c r="I90" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I90" s="8" t="inlineStr">
+      <c r="J90" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J90" s="8" t="inlineStr">
+      <c r="K90" s="8" t="inlineStr">
         <is>
           <t>Install + troubleshooting adequate.</t>
         </is>
@@ -23957,40 +24393,45 @@
       </c>
       <c r="E91" s="8" t="inlineStr">
         <is>
+          <t>P3: dedicated IG not recommended — lower/niche adoption; moderate doc gap (71.4% coverage). Prefer install how-to / API map / cross-links instead.</t>
+        </is>
+      </c>
+      <c r="F91" s="8" t="inlineStr">
+        <is>
           <t>Lower / Niche</t>
         </is>
       </c>
-      <c r="F91" s="8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
       <c r="G91" s="8" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H91" s="8" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="H91" s="8" t="inlineStr">
+      <c r="I91" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I91" s="8" t="inlineStr">
+      <c r="J91" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J91" s="8" t="inlineStr">
+      <c r="K91" s="8" t="inlineStr">
         <is>
           <t>Maintain troubleshooting; no dedicated IG beyond install.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:J91"/>
+  <autoFilter ref="A4:K91"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>